<commit_message>
Added error messages on the Login Form
</commit_message>
<xml_diff>
--- a/CustomerList.xlsx
+++ b/CustomerList.xlsx
@@ -34,6 +34,9 @@
     <x:t>Balance (₱)</x:t>
   </x:si>
   <x:si>
+    <x:t>Status</x:t>
+  </x:si>
+  <x:si>
     <x:t>6</x:t>
   </x:si>
   <x:si>
@@ -52,7 +55,10 @@
     <x:t>120.50</x:t>
   </x:si>
   <x:si>
-    <x:t>9</x:t>
+    <x:t>Active</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14</x:t>
   </x:si>
   <x:si>
     <x:t>Edwin Castro</x:t>
@@ -565,7 +571,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F12"/>
+  <x:dimension ref="A1:G12"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.996339" style="0" customWidth="1"/>
@@ -574,9 +580,10 @@
     <x:col min="4" max="4" width="12.567768" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="17.996339" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="10.567768" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:6">
+    <x:row r="1" spans="1:7">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -595,225 +602,261 @@
       <x:c r="F1" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:6">
+      <x:c r="G1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7">
       <x:c r="A2" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7">
       <x:c r="A3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:6">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:7">
       <x:c r="A4" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:7">
+      <x:c r="A5" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:6">
-      <x:c r="A5" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:6">
+      <x:c r="G5" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:7">
       <x:c r="A6" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:6">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
       <x:c r="A7" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:6">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
       <x:c r="A8" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:6">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7">
       <x:c r="A9" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:6">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:7">
       <x:c r="A10" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:6">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7">
       <x:c r="A11" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F11" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:6">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:7">
       <x:c r="A12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="G12" s="0" t="s">
+        <x:v>63</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>